<commit_message>
Incorporated domain-level ID generation, starting scaffolding for domain object factories. Updated vendor json files to include id attributes; serializers, repos all updated to include id usage. Order objects now reference vendor ids instead of names. Finally starting to set up normalization suite in core directory.
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/orders/BJ's/BJ's_Bakery_20260308.xlsx
+++ b/WorkBot/refactor-experimental/data/orders/BJ's/BJ's_Bakery_20260308.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,23 @@
       </c>
       <c r="E2" t="n">
         <v>203.94</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Celsius - Vibe Peach, Tropical, Arctic</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>28.49</v>
+      </c>
+      <c r="E3" t="n">
+        <v>199.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>